<commit_message>
added a number 4 - Commented GitLatch Commit @ 2026-4-8-17-44-9-134
</commit_message>
<xml_diff>
--- a/Test1.xlsx
+++ b/Test1.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbastard\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578E44A8-C44F-4924-B986-295D61D5FAD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7909D22E-2164-4315-BE15-14660E6E5777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{3F61093D-6EDF-4A63-A2E1-F6D5B6D08D21}"/>
   </bookViews>
@@ -402,7 +397,7 @@
   <wetp:taskpane dockstate="right" visibility="0" width="438" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="5">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -418,6 +413,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_BOARDFLARE_EXEC</we:customFunctionIds>
@@ -442,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D989ABD1-3577-4862-8836-D656AE3EE328}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -460,7 +458,13 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added a number 4 - Commented GitLatch Commit @ 2026-4-8-17-45-29-562
</commit_message>
<xml_diff>
--- a/Test1.xlsx
+++ b/Test1.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7909D22E-2164-4315-BE15-14660E6E5777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lonzagroup-my.sharepoint.com/personal/mickael_bastard_lonza_com/Documents/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B2C3BFA-70A2-4486-ACC9-2E237804CA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{3F61093D-6EDF-4A63-A2E1-F6D5B6D08D21}"/>
   </bookViews>
@@ -397,7 +402,7 @@
   <wetp:taskpane dockstate="right" visibility="0" width="438" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="511" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </wetp:taskpane>
 </wetp:taskpanes>

</xml_diff>